<commit_message>
update scenario (scenario 18 missing)
</commit_message>
<xml_diff>
--- a/scenarios_def.xlsx
+++ b/scenarios_def.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/louissallard/Desktop/ETE/Optim_JULIA/Projet/EOD-Gaz/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71A680A1-A646-7D40-AF35-E32706D234D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4954A2CD-B837-2A49-9150-265707BF6E84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4300" yWindow="5580" windowWidth="26440" windowHeight="14880" xr2:uid="{EAC5DB97-9E6B-3142-9580-796EC73B4E6C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
   <si>
     <t>Scénario</t>
   </si>
@@ -175,7 +175,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -183,6 +183,13 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1118,6 +1125,23 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
@@ -1663,8 +1687,8 @@
       <c r="B19" t="s">
         <v>20</v>
       </c>
-      <c r="C19" t="s">
-        <v>3</v>
+      <c r="C19" s="4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -1675,8 +1699,8 @@
       <c r="B20" t="s">
         <v>21</v>
       </c>
-      <c r="C20" t="s">
-        <v>3</v>
+      <c r="C20" s="4" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -1687,8 +1711,8 @@
       <c r="B21" t="s">
         <v>22</v>
       </c>
-      <c r="C21" t="s">
-        <v>3</v>
+      <c r="C21" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>27</v>
@@ -1705,8 +1729,8 @@
       <c r="B22" t="s">
         <v>23</v>
       </c>
-      <c r="C22" t="s">
-        <v>3</v>
+      <c r="C22" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="3"/>
@@ -1719,8 +1743,8 @@
       <c r="B23" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C23" t="s">
-        <v>3</v>
+      <c r="C23" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="3"/>
@@ -1733,8 +1757,8 @@
       <c r="B24" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C24" t="s">
-        <v>3</v>
+      <c r="C24" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="3"/>
@@ -1747,8 +1771,8 @@
       <c r="B25" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C25" t="s">
-        <v>3</v>
+      <c r="C25" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="3"/>

</xml_diff>